<commit_message>
z/OS 3.1 v3: B->A grade improvements (Master Catalog factual fix, +virtual-storage glossary category PSA/CSA/ECSA/SQA/ESQA/LPA/SVC/CVT, tunable kind column, default reword, 6 S-rank incident A/B/C hypothesis branching, S-rank cfg expected-output samples, scenario disclaimers per-article, image embeds 8 -> 86 entries / 57 unique). Quality gates: mkdocs strict pass.
</commit_message>
<xml_diff>
--- a/docs/products/files/zOS_3.1.xlsx
+++ b/docs/products/files/zOS_3.1.xlsx
@@ -21,6 +21,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="10_対象外項目" sheetId="12" state="visible" r:id="rId12"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="11_シナリオ別ガイド" sheetId="13" state="visible" r:id="rId13"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="12_ユースケース集" sheetId="14" state="visible" r:id="rId14"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="13_仮説分岐" sheetId="15" state="visible" r:id="rId15"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -454,7 +455,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C14"/>
+  <dimension ref="A1:C15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -606,7 +607,7 @@
       </c>
       <c r="B9" s="2" t="inlineStr">
         <is>
-          <t>45 件（オペレータ/JES2/TSO/SDSF/JCL/USS/SMP/E）</t>
+          <t>45 件</t>
         </is>
       </c>
       <c r="C9" s="2" t="inlineStr">
@@ -623,7 +624,7 @@
       </c>
       <c r="B10" s="2" t="inlineStr">
         <is>
-          <t>PARMLIB 19 メンバ + tunable 20 = 39 件</t>
+          <t>PARMLIB 19 メンバ + tunable 20</t>
         </is>
       </c>
       <c r="C10" s="2" t="inlineStr">
@@ -674,7 +675,7 @@
       </c>
       <c r="B13" s="2" t="inlineStr">
         <is>
-          <t>6 本（業務全体の俯瞰）</t>
+          <t>6 本</t>
         </is>
       </c>
       <c r="C13" s="2" t="inlineStr">
@@ -691,10 +692,27 @@
       </c>
       <c r="B14" s="2" t="inlineStr">
         <is>
-          <t>30 件（独立完結の手順）</t>
+          <t>30 件</t>
         </is>
       </c>
       <c r="C14" s="2" t="inlineStr">
+        <is>
+          <t>S_ZOS_Review</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="2" t="inlineStr">
+        <is>
+          <t>埋込図表</t>
+        </is>
+      </c>
+      <c r="B15" s="2" t="inlineStr">
+        <is>
+          <t>v3 で 73 エントリ（unique 約 57 枚）</t>
+        </is>
+      </c>
+      <c r="C15" s="2" t="inlineStr">
         <is>
           <t>S_ZOS_Review</t>
         </is>
@@ -3745,13 +3763,14 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D7"/>
+  <dimension ref="A1:E7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
   <cols>
     <col width="25" customWidth="1" min="1" max="1"/>
     <col width="50" customWidth="1" min="2" max="2"/>
-    <col width="80" customWidth="1" min="3" max="3"/>
+    <col width="60" customWidth="1" min="3" max="3"/>
     <col width="12" customWidth="1" min="4" max="4"/>
+    <col width="60" customWidth="1" min="5" max="5"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -3775,6 +3794,11 @@
           <t>本文行数</t>
         </is>
       </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>本記事の範囲</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
@@ -3795,6 +3819,11 @@
       <c r="D2" s="2" t="n">
         <v>40</v>
       </c>
+      <c r="E2" s="2" t="inlineStr">
+        <is>
+          <t>**本記事の範囲**: z/OS 新規 LPAR の初回 IPL までの PARMLIB 最低限セットを扱う。I/O 構成定義（HCD/IODF）はサイト固有のため別途 ABCs Vol.10 を参照。IBM Z ハードウェア（CPC/LPAR）の物理構成は対象外。</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
@@ -3815,6 +3844,11 @@
       <c r="D3" s="2" t="n">
         <v>21</v>
       </c>
+      <c r="E3" s="2" t="inlineStr">
+        <is>
+          <t>**本記事の範囲**: JES2 SPOOL の即時的な空き確保と中長期の容量設計を扱う。JES3 環境、NJE 経由 SYSOUT 流入の制限は対象外（個別 ABCs Vol.02 参照）。JES2 cold start を伴う SPOOLDEF 大改修は別記事 cfg-jes2-spool で扱う。</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
@@ -3835,6 +3869,11 @@
       <c r="D4" s="2" t="n">
         <v>25</v>
       </c>
+      <c r="E4" s="2" t="inlineStr">
+        <is>
+          <t>**本記事の範囲**: WLM Velocity Goal 未達の汎用切り分けフロー（RMF Mon I/III + WLM 表示）。Db2/CICS/IMS 個別の性能チューニング、Java/zCX 個別の JVM チューニングは対象外（製品マニュアル参照）。I/O 性能（Cache/HSM）は別記事の uc-rmf-io-analyze に分離。</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
@@ -3855,6 +3894,7 @@
       <c r="D5" s="2" t="n">
         <v>24</v>
       </c>
+      <c r="E5" s="2" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
@@ -3875,6 +3915,7 @@
       <c r="D6" s="2" t="n">
         <v>21</v>
       </c>
+      <c r="E6" s="2" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
@@ -3895,6 +3936,7 @@
       <c r="D7" s="2" t="n">
         <v>29</v>
       </c>
+      <c r="E7" s="2" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -4907,6 +4949,636 @@
       <c r="F31" s="2" t="inlineStr">
         <is>
           <t>cfg-grs-setup, uc-sysplex-cfrm-update</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet15.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:F19"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
+  <cols>
+    <col width="22" customWidth="1" min="1" max="1"/>
+    <col width="40" customWidth="1" min="2" max="2"/>
+    <col width="6" customWidth="1" min="3" max="3"/>
+    <col width="40" customWidth="1" min="4" max="4"/>
+    <col width="50" customWidth="1" min="5" max="5"/>
+    <col width="50" customWidth="1" min="6" max="6"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>incident ID</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>trigger</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>仮説 ID</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>仮説</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>見分け方</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>対応</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>inc-ipl-fail</t>
+        </is>
+      </c>
+      <c r="B2" s="2" t="inlineStr">
+        <is>
+          <t>z/OS が IPL 中で進まない、NIP メッセージで停止</t>
+        </is>
+      </c>
+      <c r="C2" s="2" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="D2" s="2" t="inlineStr">
+        <is>
+          <t>PARMLIB の構文エラー / 値矛盾</t>
+        </is>
+      </c>
+      <c r="E2" s="2" t="inlineStr">
+        <is>
+          <t>IEA301I / IEA302W / IEE254I 等の構文エラーメッセージが NIP に出ている</t>
+        </is>
+      </c>
+      <c r="F2" s="2" t="inlineStr">
+        <is>
+          <t>別 LOADxx で IPL → 該当メンバを ISPF EDIT → 構文修正 → 再 IPL</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="2" t="inlineStr">
+        <is>
+          <t>inc-ipl-fail</t>
+        </is>
+      </c>
+      <c r="B3" s="2" t="inlineStr">
+        <is>
+          <t>z/OS が IPL 中で進まない、NIP メッセージで停止</t>
+        </is>
+      </c>
+      <c r="C3" s="2" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="D3" s="2" t="inlineStr">
+        <is>
+          <t>IODF / I/O 構成の不整合</t>
+        </is>
+      </c>
+      <c r="E3" s="2" t="inlineStr">
+        <is>
+          <t>IOS001E / IOS118E / IGD002I 等の I/O メッセージが出る、または特定デバイスが OFFLINE</t>
+        </is>
+      </c>
+      <c r="F3" s="2" t="inlineStr">
+        <is>
+          <t>別 IODF（前世代）で IPL → HCD で IODF 修正 → ACTIVATE → 再 IPL</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="2" t="inlineStr">
+        <is>
+          <t>inc-ipl-fail</t>
+        </is>
+      </c>
+      <c r="B4" s="2" t="inlineStr">
+        <is>
+          <t>z/OS が IPL 中で進まない、NIP メッセージで停止</t>
+        </is>
+      </c>
+      <c r="C4" s="2" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="D4" s="2" t="inlineStr">
+        <is>
+          <t>Master Catalog 損傷 / SYSRES アクセス不能</t>
+        </is>
+      </c>
+      <c r="E4" s="2" t="inlineStr">
+        <is>
+          <t>IEA083E / IGW01001I 等のカタログ／VSAM エラー</t>
+        </is>
+      </c>
+      <c r="F4" s="2" t="inlineStr">
+        <is>
+          <t>Stand-Alone Restore で SYSRES 復元 → Master Catalog を IDCAMS REPRO で再構築 → IPL</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="2" t="inlineStr">
+        <is>
+          <t>inc-system-hung</t>
+        </is>
+      </c>
+      <c r="B5" s="2" t="inlineStr">
+        <is>
+          <t>z/OS 全体応答なし、コンソール反応なし</t>
+        </is>
+      </c>
+      <c r="C5" s="2" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="D5" s="2" t="inlineStr">
+        <is>
+          <t>リソース枯渇（CSA/ECSA/SQA/Aux Storage）</t>
+        </is>
+      </c>
+      <c r="E5" s="2" t="inlineStr">
+        <is>
+          <t>hung 直前に IRA200E / ILR005E / IEA602I などの容量警告が記録されている</t>
+        </is>
+      </c>
+      <c r="F5" s="2" t="inlineStr">
+        <is>
+          <t>Stand-Alone Dump → IPCS で消費 Address Space 特定 → 該当 STC 殺害 → 再 IPL 後 IEASYSxx で増量</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="2" t="inlineStr">
+        <is>
+          <t>inc-system-hung</t>
+        </is>
+      </c>
+      <c r="B6" s="2" t="inlineStr">
+        <is>
+          <t>z/OS 全体応答なし、コンソール反応なし</t>
+        </is>
+      </c>
+      <c r="C6" s="2" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="D6" s="2" t="inlineStr">
+        <is>
+          <t>デッドロック（GRS / Db2 / IMS）</t>
+        </is>
+      </c>
+      <c r="E6" s="2" t="inlineStr">
+        <is>
+          <t>D GRS,C で contention 多数、または特定 STC が長時間 WAIT</t>
+        </is>
+      </c>
+      <c r="F6" s="2" t="inlineStr">
+        <is>
+          <t>D GRS,SYSTEM,LATCH で latch holder 特定 → C/CANCEL ARM=YES で release → 必要なら SVC dump</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="2" t="inlineStr">
+        <is>
+          <t>inc-system-hung</t>
+        </is>
+      </c>
+      <c r="B7" s="2" t="inlineStr">
+        <is>
+          <t>z/OS 全体応答なし、コンソール反応なし</t>
+        </is>
+      </c>
+      <c r="C7" s="2" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="D7" s="2" t="inlineStr">
+        <is>
+          <t>ハードウェア障害（CPU / メモリ / CF link）</t>
+        </is>
+      </c>
+      <c r="E7" s="2" t="inlineStr">
+        <is>
+          <t>HMC SE で hardware error log（PCHID error 等）が出ている</t>
+        </is>
+      </c>
+      <c r="F7" s="2" t="inlineStr">
+        <is>
+          <t>HMC で hardware status 確認 → IBM ハードウェアサポートへ。回避は別 LPAR への workload 移動</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="2" t="inlineStr">
+        <is>
+          <t>inc-jes2-spool-full</t>
+        </is>
+      </c>
+      <c r="B8" s="2" t="inlineStr">
+        <is>
+          <t>$HASP050 SHORT ON SPOOL SPACE 発生、新規ジョブ受付不能</t>
+        </is>
+      </c>
+      <c r="C8" s="2" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="D8" s="2" t="inlineStr">
+        <is>
+          <t>完了済ジョブの蓄積（HOLD class 等で purge されていない）</t>
+        </is>
+      </c>
+      <c r="E8" s="2" t="inlineStr">
+        <is>
+          <t>$D Q で大量の OUTPUT/HOLD ジョブ、SDSF H で hold 数が多い</t>
+        </is>
+      </c>
+      <c r="F8" s="2" t="inlineStr">
+        <is>
+          <t>SDSF ST → 不要ジョブ P でパージ。SDSF H → P で hardcopy パージ。$T &lt;CLASS&gt;,OUTPUT=PURGE で自動化検討</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="2" t="inlineStr">
+        <is>
+          <t>inc-jes2-spool-full</t>
+        </is>
+      </c>
+      <c r="B9" s="2" t="inlineStr">
+        <is>
+          <t>$HASP050 SHORT ON SPOOL SPACE 発生、新規ジョブ受付不能</t>
+        </is>
+      </c>
+      <c r="C9" s="2" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="D9" s="2" t="inlineStr">
+        <is>
+          <t>暴走ジョブによる SYSOUT 大量出力</t>
+        </is>
+      </c>
+      <c r="E9" s="2" t="inlineStr">
+        <is>
+          <t>$D Q で特定ジョブの SYSOUT サイズが異常</t>
+        </is>
+      </c>
+      <c r="F9" s="2" t="inlineStr">
+        <is>
+          <t>$C &lt;jobid&gt; でジョブキャンセル → SYSOUT パージ → アプリケーション側で OUTLIM 等の上限設定</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="2" t="inlineStr">
+        <is>
+          <t>inc-jes2-spool-full</t>
+        </is>
+      </c>
+      <c r="B10" s="2" t="inlineStr">
+        <is>
+          <t>$HASP050 SHORT ON SPOOL SPACE 発生、新規ジョブ受付不能</t>
+        </is>
+      </c>
+      <c r="C10" s="2" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="D10" s="2" t="inlineStr">
+        <is>
+          <t>SPOOL volume 容量設計の限界</t>
+        </is>
+      </c>
+      <c r="E10" s="2" t="inlineStr">
+        <is>
+          <t>$D SPL で全 volume の利用率が均等に高い、定常状態での増加</t>
+        </is>
+      </c>
+      <c r="F10" s="2" t="inlineStr">
+        <is>
+          <t>$T SPOOL ADD で新規 SPOOL volume 追加（DASD 事前確保必要）。中長期で cold start で SPOOLDEF 拡張</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="2" t="inlineStr">
+        <is>
+          <t>inc-paging-shortage</t>
+        </is>
+      </c>
+      <c r="B11" s="2" t="inlineStr">
+        <is>
+          <t>ILR005E AUXILIARY STORAGE SHORTAGE</t>
+        </is>
+      </c>
+      <c r="C11" s="2" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="D11" s="2" t="inlineStr">
+        <is>
+          <t>メモリリーク STC が大量 paging を発生させている</t>
+        </is>
+      </c>
+      <c r="E11" s="2" t="inlineStr">
+        <is>
+          <t>D ASM,PLPA で PLPA は正常、LOCAL のみ高使用。RMF Mon III で特定 ASID が常に high working set</t>
+        </is>
+      </c>
+      <c r="F11" s="2" t="inlineStr">
+        <is>
+          <t>該当 STC を P で停止 → 起動元の保守 PTF 確認</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="2" t="inlineStr">
+        <is>
+          <t>inc-paging-shortage</t>
+        </is>
+      </c>
+      <c r="B12" s="2" t="inlineStr">
+        <is>
+          <t>ILR005E AUXILIARY STORAGE SHORTAGE</t>
+        </is>
+      </c>
+      <c r="C12" s="2" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="D12" s="2" t="inlineStr">
+        <is>
+          <t>突発負荷で正常なバッチが paging を引き起こす</t>
+        </is>
+      </c>
+      <c r="E12" s="2" t="inlineStr">
+        <is>
+          <t>JES2 で同時 active job 数が異常に多い</t>
+        </is>
+      </c>
+      <c r="F12" s="2" t="inlineStr">
+        <is>
+          <t>$P INIT で initiator 数を一時減少 → 完了待ち → 段階的に復帰</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="2" t="inlineStr">
+        <is>
+          <t>inc-paging-shortage</t>
+        </is>
+      </c>
+      <c r="B13" s="2" t="inlineStr">
+        <is>
+          <t>ILR005E AUXILIARY STORAGE SHORTAGE</t>
+        </is>
+      </c>
+      <c r="C13" s="2" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="D13" s="2" t="inlineStr">
+        <is>
+          <t>ページデータセット容量設計不足</t>
+        </is>
+      </c>
+      <c r="E13" s="2" t="inlineStr">
+        <is>
+          <t>D ASM で全タイプ（PLPA/COMMON/LOCAL）が定常的に高使用率</t>
+        </is>
+      </c>
+      <c r="F13" s="2" t="inlineStr">
+        <is>
+          <t>PAGEADD で新規 LOCAL ページデータセット動的追加 → 中長期で IEASYSxx PAGE= 拡張</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="2" t="inlineStr">
+        <is>
+          <t>inc-tcpip-down</t>
+        </is>
+      </c>
+      <c r="B14" s="2" t="inlineStr">
+        <is>
+          <t>TCP/IP 通信不能、ping 失敗</t>
+        </is>
+      </c>
+      <c r="C14" s="2" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="D14" s="2" t="inlineStr">
+        <is>
+          <t>TCPIP STC 自体が down/hung</t>
+        </is>
+      </c>
+      <c r="E14" s="2" t="inlineStr">
+        <is>
+          <t>D A,L で TCPIP が ACTIVE でない、または応答なし</t>
+        </is>
+      </c>
+      <c r="F14" s="2" t="inlineStr">
+        <is>
+          <t>TCPIP STC を P → S で再起動。hung なら C → S。NETSTAT 取得不能で確認</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="2" t="inlineStr">
+        <is>
+          <t>inc-tcpip-down</t>
+        </is>
+      </c>
+      <c r="B15" s="2" t="inlineStr">
+        <is>
+          <t>TCP/IP 通信不能、ping 失敗</t>
+        </is>
+      </c>
+      <c r="C15" s="2" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="D15" s="2" t="inlineStr">
+        <is>
+          <t>ネットワークインターフェース（OSA/HiperSocket）障害</t>
+        </is>
+      </c>
+      <c r="E15" s="2" t="inlineStr">
+        <is>
+          <t>NETSTAT DEV で OSA インターフェースが INACTIVE / NOT ACTIVE</t>
+        </is>
+      </c>
+      <c r="F15" s="2" t="inlineStr">
+        <is>
+          <t>VARY OBEY で device 再活性化、HMC で OSA hardware status 確認</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="2" t="inlineStr">
+        <is>
+          <t>inc-tcpip-down</t>
+        </is>
+      </c>
+      <c r="B16" s="2" t="inlineStr">
+        <is>
+          <t>TCP/IP 通信不能、ping 失敗</t>
+        </is>
+      </c>
+      <c r="C16" s="2" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="D16" s="2" t="inlineStr">
+        <is>
+          <t>PROFILE.TCPIP 設定誤り（HOME / ROUTE / GATEWAY）</t>
+        </is>
+      </c>
+      <c r="E16" s="2" t="inlineStr">
+        <is>
+          <t>NETSTAT HOME で HOME IP 不在、NETSTAT ROUTE で default route 不在</t>
+        </is>
+      </c>
+      <c r="F16" s="2" t="inlineStr">
+        <is>
+          <t>PROFILE.TCPIP 修正 → V TCPIP,,OBEYFILE で動的反映 → ping 再試行</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="2" t="inlineStr">
+        <is>
+          <t>inc-racf-access-denied</t>
+        </is>
+      </c>
+      <c r="B17" s="2" t="inlineStr">
+        <is>
+          <t>ICH408I INSUFFICIENT ACCESS AUTHORITY</t>
+        </is>
+      </c>
+      <c r="C17" s="2" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="D17" s="2" t="inlineStr">
+        <is>
+          <t>プロファイルに対する権限不足（PERMIT 不在）</t>
+        </is>
+      </c>
+      <c r="E17" s="2" t="inlineStr">
+        <is>
+          <t>RLIST &lt;class&gt; '&lt;profile&gt;' AUTHUSER で対象ユーザの ACCESS 列が NONE / READ 不足</t>
+        </is>
+      </c>
+      <c r="F17" s="2" t="inlineStr">
+        <is>
+          <t>PERMIT '&lt;profile&gt;' CLASS(&lt;class&gt;) ID(&lt;user&gt;) ACCESS(&lt;level&gt;) → SETR REFRESH</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="2" t="inlineStr">
+        <is>
+          <t>inc-racf-access-denied</t>
+        </is>
+      </c>
+      <c r="B18" s="2" t="inlineStr">
+        <is>
+          <t>ICH408I INSUFFICIENT ACCESS AUTHORITY</t>
+        </is>
+      </c>
+      <c r="C18" s="2" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="D18" s="2" t="inlineStr">
+        <is>
+          <t>プロファイル自体がない（UACC NONE 状態）</t>
+        </is>
+      </c>
+      <c r="E18" s="2" t="inlineStr">
+        <is>
+          <t>RLIST &lt;class&gt; '&lt;profile&gt;' で NOT FOUND</t>
+        </is>
+      </c>
+      <c r="F18" s="2" t="inlineStr">
+        <is>
+          <t>RDEFINE &lt;class&gt; '&lt;profile&gt;' UACC(NONE) AUDIT(SUCCESS,FAILURES) → PERMIT で個別権限</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="2" t="inlineStr">
+        <is>
+          <t>inc-racf-access-denied</t>
+        </is>
+      </c>
+      <c r="B19" s="2" t="inlineStr">
+        <is>
+          <t>ICH408I INSUFFICIENT ACCESS AUTHORITY</t>
+        </is>
+      </c>
+      <c r="C19" s="2" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="D19" s="2" t="inlineStr">
+        <is>
+          <t>GENERIC プロファイルの REFRESH 漏れ</t>
+        </is>
+      </c>
+      <c r="E19" s="2" t="inlineStr">
+        <is>
+          <t>PERMIT 直後で SETR REFRESH 未実施、GENERIC class（DATASET 等）で発生</t>
+        </is>
+      </c>
+      <c r="F19" s="2" t="inlineStr">
+        <is>
+          <t>SETROPTS GENERIC(&lt;class&gt;) REFRESH → 再アクセステスト</t>
         </is>
       </c>
     </row>
@@ -7939,18 +8611,19 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I21"/>
+  <dimension ref="A1:J21"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
-    <col width="30" customWidth="1" min="2" max="2"/>
-    <col width="35" customWidth="1" min="3" max="3"/>
+    <col width="14" customWidth="1" min="2" max="2"/>
+    <col width="30" customWidth="1" min="3" max="3"/>
     <col width="35" customWidth="1" min="4" max="4"/>
     <col width="35" customWidth="1" min="5" max="5"/>
-    <col width="22" customWidth="1" min="6" max="6"/>
+    <col width="35" customWidth="1" min="6" max="6"/>
     <col width="22" customWidth="1" min="7" max="7"/>
-    <col width="16" customWidth="1" min="8" max="8"/>
-    <col width="35" customWidth="1" min="9" max="9"/>
+    <col width="22" customWidth="1" min="8" max="8"/>
+    <col width="16" customWidth="1" min="9" max="9"/>
+    <col width="35" customWidth="1" min="10" max="10"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -7961,40 +8634,45 @@
       </c>
       <c r="B1" s="1" t="inlineStr">
         <is>
+          <t>種別</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
           <t>設定コマンド</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="D1" s="1" t="inlineStr">
         <is>
           <t>デフォルト</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="E1" s="1" t="inlineStr">
         <is>
           <t>取り得る値</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="F1" s="1" t="inlineStr">
         <is>
           <t>影響範囲</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="G1" s="1" t="inlineStr">
         <is>
           <t>関連</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
+      <c r="H1" s="1" t="inlineStr">
         <is>
           <t>関連手順</t>
         </is>
       </c>
-      <c r="H1" s="1" t="inlineStr">
+      <c r="I1" s="1" t="inlineStr">
         <is>
           <t>出典</t>
         </is>
       </c>
-      <c r="I1" s="1" t="inlineStr">
+      <c r="J1" s="1" t="inlineStr">
         <is>
           <t>注意点</t>
         </is>
@@ -8008,40 +8686,45 @@
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
+          <t>サイジング</t>
+        </is>
+      </c>
+      <c r="C2" s="2" t="inlineStr">
+        <is>
           <t>BPXPRMxx</t>
         </is>
       </c>
-      <c r="C2" s="2" t="inlineStr">
+      <c r="D2" s="2" t="inlineStr">
         <is>
           <t>2147483647（≒ 2GB-1）</t>
         </is>
       </c>
-      <c r="D2" s="2" t="inlineStr">
+      <c r="E2" s="2" t="inlineStr">
         <is>
           <t>0〜2147483647（バイト）</t>
         </is>
       </c>
-      <c r="E2" s="2" t="inlineStr">
+      <c r="F2" s="2" t="inlineStr">
         <is>
           <t>次回 IPL or SET OMVS=xx で動的反映</t>
         </is>
       </c>
-      <c r="F2" s="2" t="inlineStr">
+      <c r="G2" s="2" t="inlineStr">
         <is>
           <t>USS, MAXSHAREPAGES</t>
         </is>
       </c>
-      <c r="G2" s="2" t="inlineStr">
+      <c r="H2" s="2" t="inlineStr">
         <is>
           <t>cfg-uss-fs</t>
         </is>
       </c>
-      <c r="H2" s="2" t="inlineStr">
+      <c r="I2" s="2" t="inlineStr">
         <is>
           <t>S_ZOS_USS</t>
         </is>
       </c>
-      <c r="I2" s="2" t="inlineStr">
+      <c r="J2" s="2" t="inlineStr">
         <is>
           <t>USS プロセスの最大 address space サイズ。Java 等の大規模アプリでは 4GB 以上推奨。</t>
         </is>
@@ -8055,40 +8738,45 @@
       </c>
       <c r="B3" s="2" t="inlineStr">
         <is>
+          <t>サイジング</t>
+        </is>
+      </c>
+      <c r="C3" s="2" t="inlineStr">
+        <is>
           <t>BPXPRMxx</t>
         </is>
       </c>
-      <c r="C3" s="2" t="inlineStr">
+      <c r="D3" s="2" t="inlineStr">
         <is>
           <t>64000</t>
         </is>
       </c>
-      <c r="D3" s="2" t="inlineStr">
+      <c r="E3" s="2" t="inlineStr">
         <is>
           <t>1〜524287</t>
         </is>
       </c>
-      <c r="E3" s="2" t="inlineStr">
+      <c r="F3" s="2" t="inlineStr">
         <is>
           <t>次回 IPL or SET OMVS=xx</t>
         </is>
       </c>
-      <c r="F3" s="2" t="inlineStr">
+      <c r="G3" s="2" t="inlineStr">
         <is>
           <t>USS, ulimit -n</t>
         </is>
       </c>
-      <c r="G3" s="2" t="inlineStr">
+      <c r="H3" s="2" t="inlineStr">
         <is>
           <t>cfg-uss-fs</t>
         </is>
       </c>
-      <c r="H3" s="2" t="inlineStr">
+      <c r="I3" s="2" t="inlineStr">
         <is>
           <t>S_ZOS_USS</t>
         </is>
       </c>
-      <c r="I3" s="2" t="inlineStr">
+      <c r="J3" s="2" t="inlineStr">
         <is>
           <t>USS プロセスあたりの最大オープンファイル数。Web/DB サーバで増量必要なケース多い。</t>
         </is>
@@ -8102,40 +8790,45 @@
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
+          <t>サイジング</t>
+        </is>
+      </c>
+      <c r="C4" s="2" t="inlineStr">
+        <is>
           <t>BPXPRMxx</t>
         </is>
       </c>
-      <c r="C4" s="2" t="inlineStr">
+      <c r="D4" s="2" t="inlineStr">
         <is>
           <t>200</t>
         </is>
       </c>
-      <c r="D4" s="2" t="inlineStr">
+      <c r="E4" s="2" t="inlineStr">
         <is>
           <t>0〜100000</t>
         </is>
       </c>
-      <c r="E4" s="2" t="inlineStr">
+      <c r="F4" s="2" t="inlineStr">
         <is>
           <t>次回 IPL or SET OMVS=xx</t>
         </is>
       </c>
-      <c r="F4" s="2" t="inlineStr">
+      <c r="G4" s="2" t="inlineStr">
         <is>
           <t>USS, MAXTHREADTASKS</t>
         </is>
       </c>
-      <c r="G4" s="2" t="inlineStr">
+      <c r="H4" s="2" t="inlineStr">
         <is>
           <t>cfg-uss-fs</t>
         </is>
       </c>
-      <c r="H4" s="2" t="inlineStr">
+      <c r="I4" s="2" t="inlineStr">
         <is>
           <t>S_ZOS_USS</t>
         </is>
       </c>
-      <c r="I4" s="2" t="inlineStr">
+      <c r="J4" s="2" t="inlineStr">
         <is>
           <t>USS プロセスあたりの最大スレッド数。Java application server で増量推奨。</t>
         </is>
@@ -8149,40 +8842,45 @@
       </c>
       <c r="B5" s="2" t="inlineStr">
         <is>
+          <t>構成定義</t>
+        </is>
+      </c>
+      <c r="C5" s="2" t="inlineStr">
+        <is>
           <t>SMFPRMxx の TYPE() オペランド</t>
         </is>
       </c>
-      <c r="C5" s="2" t="inlineStr">
+      <c r="D5" s="2" t="inlineStr">
         <is>
           <t>サイトにより異なる（典型 0,30,42,70-79,80,89,90,99 等）</t>
         </is>
       </c>
-      <c r="D5" s="2" t="inlineStr">
+      <c r="E5" s="2" t="inlineStr">
         <is>
           <t>0-255 の任意組み合わせ</t>
         </is>
       </c>
-      <c r="E5" s="2" t="inlineStr">
+      <c r="F5" s="2" t="inlineStr">
         <is>
           <t>SET SMF=xx で動的反映</t>
         </is>
       </c>
-      <c r="F5" s="2" t="inlineStr">
+      <c r="G5" s="2" t="inlineStr">
         <is>
           <t>SMF</t>
         </is>
       </c>
-      <c r="G5" s="2" t="inlineStr">
+      <c r="H5" s="2" t="inlineStr">
         <is>
           <t>cfg-smf-collect</t>
         </is>
       </c>
-      <c r="H5" s="2" t="inlineStr">
+      <c r="I5" s="2" t="inlineStr">
         <is>
           <t>S_ZOS_SMF</t>
         </is>
       </c>
-      <c r="I5" s="2" t="inlineStr">
+      <c r="J5" s="2" t="inlineStr">
         <is>
           <t>TYPE 30 = ジョブ統計、80 = RACF、70-79 = RMF、89 = USS、99 = WLM。</t>
         </is>
@@ -8196,40 +8894,45 @@
       </c>
       <c r="B6" s="2" t="inlineStr">
         <is>
+          <t>サイジング</t>
+        </is>
+      </c>
+      <c r="C6" s="2" t="inlineStr">
+        <is>
           <t>IEASYSxx の CSA= オペランド</t>
         </is>
       </c>
-      <c r="C6" s="2" t="inlineStr">
+      <c r="D6" s="2" t="inlineStr">
         <is>
           <t>サイトにより異なる（例: 256M）</t>
         </is>
       </c>
-      <c r="D6" s="2" t="inlineStr">
+      <c r="E6" s="2" t="inlineStr">
         <is>
           <t>0M〜2047M</t>
         </is>
       </c>
-      <c r="E6" s="2" t="inlineStr">
+      <c r="F6" s="2" t="inlineStr">
         <is>
           <t>次回 IPL 時のみ</t>
         </is>
       </c>
-      <c r="F6" s="2" t="inlineStr">
+      <c r="G6" s="2" t="inlineStr">
         <is>
           <t>ECSA, SQA</t>
         </is>
       </c>
-      <c r="G6" s="2" t="inlineStr">
+      <c r="H6" s="2" t="inlineStr">
         <is>
           <t>cfg-parmlib-update</t>
         </is>
       </c>
-      <c r="H6" s="2" t="inlineStr">
+      <c r="I6" s="2" t="inlineStr">
         <is>
           <t>S_ZOS_Init_Tuning</t>
         </is>
       </c>
-      <c r="I6" s="2" t="inlineStr">
+      <c r="J6" s="2" t="inlineStr">
         <is>
           <t>Common Storage Area サイズ。アプリ要件で増減。</t>
         </is>
@@ -8243,40 +8946,45 @@
       </c>
       <c r="B7" s="2" t="inlineStr">
         <is>
+          <t>サイジング</t>
+        </is>
+      </c>
+      <c r="C7" s="2" t="inlineStr">
+        <is>
           <t>IEASYSxx の CSA= で 2 番目の値</t>
         </is>
       </c>
-      <c r="C7" s="2" t="inlineStr">
+      <c r="D7" s="2" t="inlineStr">
         <is>
           <t>サイトにより異なる（例: 1024M）</t>
         </is>
       </c>
-      <c r="D7" s="2" t="inlineStr">
+      <c r="E7" s="2" t="inlineStr">
         <is>
           <t>0M〜2047M</t>
         </is>
       </c>
-      <c r="E7" s="2" t="inlineStr">
+      <c r="F7" s="2" t="inlineStr">
         <is>
           <t>次回 IPL 時のみ</t>
         </is>
       </c>
-      <c r="F7" s="2" t="inlineStr">
+      <c r="G7" s="2" t="inlineStr">
         <is>
           <t>CSAALOC</t>
         </is>
       </c>
-      <c r="G7" s="2" t="inlineStr">
+      <c r="H7" s="2" t="inlineStr">
         <is>
           <t>cfg-parmlib-update</t>
         </is>
       </c>
-      <c r="H7" s="2" t="inlineStr">
+      <c r="I7" s="2" t="inlineStr">
         <is>
           <t>S_ZOS_Init_Tuning</t>
         </is>
       </c>
-      <c r="I7" s="2" t="inlineStr">
+      <c r="J7" s="2" t="inlineStr">
         <is>
           <t>Extended CSA。16MB 境界より上の CSA。多くのサブシステム（Db2, CICS）が消費。</t>
         </is>
@@ -8290,40 +8998,45 @@
       </c>
       <c r="B8" s="2" t="inlineStr">
         <is>
+          <t>モード選択</t>
+        </is>
+      </c>
+      <c r="C8" s="2" t="inlineStr">
+        <is>
           <t>IEASYSxx の GRS= オペランド</t>
         </is>
       </c>
-      <c r="C8" s="2" t="inlineStr">
-        <is>
-          <t>STAR（Sysplex 環境）</t>
-        </is>
-      </c>
       <c r="D8" s="2" t="inlineStr">
         <is>
+          <t>STAR モード（Sysplex 環境の標準値、CF 経由 Lock 構造）</t>
+        </is>
+      </c>
+      <c r="E8" s="2" t="inlineStr">
+        <is>
           <t>NONE / RING / STAR</t>
         </is>
       </c>
-      <c r="E8" s="2" t="inlineStr">
+      <c r="F8" s="2" t="inlineStr">
         <is>
           <t>次回 IPL 時のみ</t>
         </is>
       </c>
-      <c r="F8" s="2" t="inlineStr">
+      <c r="G8" s="2" t="inlineStr">
         <is>
           <t>GRS, GRSRNLxx</t>
         </is>
       </c>
-      <c r="G8" s="2" t="inlineStr">
+      <c r="H8" s="2" t="inlineStr">
         <is>
           <t>cfg-grs-setup</t>
         </is>
       </c>
-      <c r="H8" s="2" t="inlineStr">
+      <c r="I8" s="2" t="inlineStr">
         <is>
           <t>S_ZOS_Sysplex</t>
         </is>
       </c>
-      <c r="I8" s="2" t="inlineStr">
+      <c r="J8" s="2" t="inlineStr">
         <is>
           <t>Sysplex 環境では STAR 必須。CF を介した Lock 構造で性能向上。</t>
         </is>
@@ -8337,40 +9050,45 @@
       </c>
       <c r="B9" s="2" t="inlineStr">
         <is>
+          <t>モード選択</t>
+        </is>
+      </c>
+      <c r="C9" s="2" t="inlineStr">
+        <is>
           <t>IEASYSxx の CLPA</t>
         </is>
       </c>
-      <c r="C9" s="2" t="inlineStr">
-        <is>
-          <t>（なし）= 既存 LPA を再利用</t>
-        </is>
-      </c>
       <c r="D9" s="2" t="inlineStr">
         <is>
+          <t>（指定なし = 既存 LPA キャッシュを再利用、CLPA 指定で再構築）</t>
+        </is>
+      </c>
+      <c r="E9" s="2" t="inlineStr">
+        <is>
           <t>CLPA 指定 or 不指定</t>
         </is>
       </c>
-      <c r="E9" s="2" t="inlineStr">
+      <c r="F9" s="2" t="inlineStr">
         <is>
           <t>次回 IPL 時のみ</t>
         </is>
       </c>
-      <c r="F9" s="2" t="inlineStr">
+      <c r="G9" s="2" t="inlineStr">
         <is>
           <t>LPA, LPALSTxx</t>
         </is>
       </c>
-      <c r="G9" s="2" t="inlineStr">
+      <c r="H9" s="2" t="inlineStr">
         <is>
           <t>cfg-clpa-ipl</t>
         </is>
       </c>
-      <c r="H9" s="2" t="inlineStr">
+      <c r="I9" s="2" t="inlineStr">
         <is>
           <t>S_ZOS_Init_Tuning</t>
         </is>
       </c>
-      <c r="I9" s="2" t="inlineStr">
+      <c r="J9" s="2" t="inlineStr">
         <is>
           <t>LPALIB から LPA 再構築。常駐モジュール変更 / メンテ後に必要。</t>
         </is>
@@ -8384,40 +9102,45 @@
       </c>
       <c r="B10" s="2" t="inlineStr">
         <is>
+          <t>構成定義</t>
+        </is>
+      </c>
+      <c r="C10" s="2" t="inlineStr">
+        <is>
           <t>JES2 INITDECK の JOBCLASS(x)</t>
         </is>
       </c>
-      <c r="C10" s="2" t="inlineStr">
+      <c r="D10" s="2" t="inlineStr">
         <is>
           <t>サイトにより異なる</t>
         </is>
       </c>
-      <c r="D10" s="2" t="inlineStr">
+      <c r="E10" s="2" t="inlineStr">
         <is>
           <t>JOBCLASS(A)〜JOBCLASS(9)</t>
         </is>
       </c>
-      <c r="E10" s="2" t="inlineStr">
+      <c r="F10" s="2" t="inlineStr">
         <is>
           <t>$T JOBCLASS(x),... で動的変更</t>
         </is>
       </c>
-      <c r="F10" s="2" t="inlineStr">
+      <c r="G10" s="2" t="inlineStr">
         <is>
           <t>JES2 Class, Initiator</t>
         </is>
       </c>
-      <c r="G10" s="2" t="inlineStr">
+      <c r="H10" s="2" t="inlineStr">
         <is>
           <t>cfg-jes2-init</t>
         </is>
       </c>
-      <c r="H10" s="2" t="inlineStr">
+      <c r="I10" s="2" t="inlineStr">
         <is>
           <t>S_ZOS_JES2</t>
         </is>
       </c>
-      <c r="I10" s="2" t="inlineStr">
+      <c r="J10" s="2" t="inlineStr">
         <is>
           <t>クラスごとに優先度・MAXJOBS 等を設定。CLASS=A は通常運用、TSU は TSO 専用。</t>
         </is>
@@ -8431,40 +9154,45 @@
       </c>
       <c r="B11" s="2" t="inlineStr">
         <is>
+          <t>構成定義</t>
+        </is>
+      </c>
+      <c r="C11" s="2" t="inlineStr">
+        <is>
           <t>JES2 INITDECK の INITDEF</t>
         </is>
       </c>
-      <c r="C11" s="2" t="inlineStr">
+      <c r="D11" s="2" t="inlineStr">
         <is>
           <t>サイトにより異なる</t>
         </is>
       </c>
-      <c r="D11" s="2" t="inlineStr">
+      <c r="E11" s="2" t="inlineStr">
         <is>
           <t>1〜100 のイニシエータ数</t>
         </is>
       </c>
-      <c r="E11" s="2" t="inlineStr">
+      <c r="F11" s="2" t="inlineStr">
         <is>
           <t>JES2 warm/cold start。$S I, $P I で動的開始/停止</t>
         </is>
       </c>
-      <c r="F11" s="2" t="inlineStr">
+      <c r="G11" s="2" t="inlineStr">
         <is>
           <t>JES2 Initiator, JOBCLASS</t>
         </is>
       </c>
-      <c r="G11" s="2" t="inlineStr">
+      <c r="H11" s="2" t="inlineStr">
         <is>
           <t>cfg-jes2-init</t>
         </is>
       </c>
-      <c r="H11" s="2" t="inlineStr">
+      <c r="I11" s="2" t="inlineStr">
         <is>
           <t>S_ZOS_JES2</t>
         </is>
       </c>
-      <c r="I11" s="2" t="inlineStr">
+      <c r="J11" s="2" t="inlineStr">
         <is>
           <t>INITDEF=10,A,B 等で 10 個のイニシエータを Class A,B 受け持ちで定義。</t>
         </is>
@@ -8478,40 +9206,45 @@
       </c>
       <c r="B12" s="2" t="inlineStr">
         <is>
+          <t>構成定義</t>
+        </is>
+      </c>
+      <c r="C12" s="2" t="inlineStr">
+        <is>
           <t>JES2 INITDECK の SPOOLDEF</t>
         </is>
       </c>
-      <c r="C12" s="2" t="inlineStr">
+      <c r="D12" s="2" t="inlineStr">
         <is>
           <t>サイトにより異なる</t>
         </is>
       </c>
-      <c r="D12" s="2" t="inlineStr">
+      <c r="E12" s="2" t="inlineStr">
         <is>
           <t>VOLSER, BUFSIZE 等</t>
         </is>
       </c>
-      <c r="E12" s="2" t="inlineStr">
+      <c r="F12" s="2" t="inlineStr">
         <is>
           <t>JES2 cold start のみ</t>
         </is>
       </c>
-      <c r="F12" s="2" t="inlineStr">
+      <c r="G12" s="2" t="inlineStr">
         <is>
           <t>JES2 SPOOL</t>
         </is>
       </c>
-      <c r="G12" s="2" t="inlineStr">
+      <c r="H12" s="2" t="inlineStr">
         <is>
           <t>cfg-jes2-spool</t>
         </is>
       </c>
-      <c r="H12" s="2" t="inlineStr">
+      <c r="I12" s="2" t="inlineStr">
         <is>
           <t>S_ZOS_JES2</t>
         </is>
       </c>
-      <c r="I12" s="2" t="inlineStr">
+      <c r="J12" s="2" t="inlineStr">
         <is>
           <t>SPOOL volume 追加時は cold start 必要 or $T で hot add（条件あり）。</t>
         </is>
@@ -8525,40 +9258,45 @@
       </c>
       <c r="B13" s="2" t="inlineStr">
         <is>
+          <t>運用ポリシー</t>
+        </is>
+      </c>
+      <c r="C13" s="2" t="inlineStr">
+        <is>
           <t>WLM Service Class 定義</t>
         </is>
       </c>
-      <c r="C13" s="2" t="inlineStr">
+      <c r="D13" s="2" t="inlineStr">
         <is>
           <t>サイトにより異なる</t>
         </is>
       </c>
-      <c r="D13" s="2" t="inlineStr">
+      <c r="E13" s="2" t="inlineStr">
         <is>
           <t>1〜99（%）</t>
         </is>
       </c>
-      <c r="E13" s="2" t="inlineStr">
+      <c r="F13" s="2" t="inlineStr">
         <is>
           <t>WLM POLICY ACTIVATE で動的</t>
         </is>
       </c>
-      <c r="F13" s="2" t="inlineStr">
+      <c r="G13" s="2" t="inlineStr">
         <is>
           <t>WLM, Service Class</t>
         </is>
       </c>
-      <c r="G13" s="2" t="inlineStr">
+      <c r="H13" s="2" t="inlineStr">
         <is>
           <t>cfg-wlm-policy</t>
         </is>
       </c>
-      <c r="H13" s="2" t="inlineStr">
+      <c r="I13" s="2" t="inlineStr">
         <is>
           <t>S_ZOS_WLM</t>
         </is>
       </c>
-      <c r="I13" s="2" t="inlineStr">
+      <c r="J13" s="2" t="inlineStr">
         <is>
           <t>Velocity = (CPU using) / (CPU using + delays) %。バッチで 30〜60、STC で 70〜90 が一般的（要 IBM Sizing Guide 確認）。</t>
         </is>
@@ -8572,40 +9310,45 @@
       </c>
       <c r="B14" s="2" t="inlineStr">
         <is>
+          <t>運用ポリシー</t>
+        </is>
+      </c>
+      <c r="C14" s="2" t="inlineStr">
+        <is>
           <t>WLM Service Class 定義</t>
         </is>
       </c>
-      <c r="C14" s="2" t="inlineStr">
+      <c r="D14" s="2" t="inlineStr">
         <is>
           <t>サイトにより異なる</t>
         </is>
       </c>
-      <c r="D14" s="2" t="inlineStr">
+      <c r="E14" s="2" t="inlineStr">
         <is>
           <t>ms / sec</t>
         </is>
       </c>
-      <c r="E14" s="2" t="inlineStr">
+      <c r="F14" s="2" t="inlineStr">
         <is>
           <t>WLM POLICY ACTIVATE</t>
         </is>
       </c>
-      <c r="F14" s="2" t="inlineStr">
+      <c r="G14" s="2" t="inlineStr">
         <is>
           <t>WLM, Service Class</t>
         </is>
       </c>
-      <c r="G14" s="2" t="inlineStr">
+      <c r="H14" s="2" t="inlineStr">
         <is>
           <t>cfg-wlm-policy</t>
         </is>
       </c>
-      <c r="H14" s="2" t="inlineStr">
+      <c r="I14" s="2" t="inlineStr">
         <is>
           <t>S_ZOS_WLM</t>
         </is>
       </c>
-      <c r="I14" s="2" t="inlineStr">
+      <c r="J14" s="2" t="inlineStr">
         <is>
           <t>Average Response Time / Percentile Response Time の 2 種。CICS/IMS 等の対話業務で使用。</t>
         </is>
@@ -8619,40 +9362,45 @@
       </c>
       <c r="B15" s="2" t="inlineStr">
         <is>
+          <t>構成定義</t>
+        </is>
+      </c>
+      <c r="C15" s="2" t="inlineStr">
+        <is>
           <t>CONSOLxx の AUTH() オペランド</t>
         </is>
       </c>
-      <c r="C15" s="2" t="inlineStr">
-        <is>
-          <t>INFO（最小権限）</t>
-        </is>
-      </c>
       <c r="D15" s="2" t="inlineStr">
         <is>
+          <t>INFO（最小権限。コマンド入力可・システム影響なし）</t>
+        </is>
+      </c>
+      <c r="E15" s="2" t="inlineStr">
+        <is>
           <t>INFO / SYS / IO / CONS / MASTER</t>
         </is>
       </c>
-      <c r="E15" s="2" t="inlineStr">
+      <c r="F15" s="2" t="inlineStr">
         <is>
           <t>次回 IPL or VARY CN</t>
         </is>
       </c>
-      <c r="F15" s="2" t="inlineStr">
+      <c r="G15" s="2" t="inlineStr">
         <is>
           <t>Console</t>
         </is>
       </c>
-      <c r="G15" s="2" t="inlineStr">
+      <c r="H15" s="2" t="inlineStr">
         <is>
           <t>cfg-console-add</t>
         </is>
       </c>
-      <c r="H15" s="2" t="inlineStr">
+      <c r="I15" s="2" t="inlineStr">
         <is>
           <t>S_ZOS_MVS_Init</t>
         </is>
       </c>
-      <c r="I15" s="2" t="inlineStr">
+      <c r="J15" s="2" t="inlineStr">
         <is>
           <t>MASTER 権限のコンソールは重要オペレータコマンド発行可能。RACF 連携でユーザ単位制御も可能。</t>
         </is>
@@ -8666,40 +9414,45 @@
       </c>
       <c r="B16" s="2" t="inlineStr">
         <is>
+          <t>サイジング</t>
+        </is>
+      </c>
+      <c r="C16" s="2" t="inlineStr">
+        <is>
           <t>PROFILE.TCPIP の TCPCONFIG MAXSOCK</t>
         </is>
       </c>
-      <c r="C16" s="2" t="inlineStr">
+      <c r="D16" s="2" t="inlineStr">
         <is>
           <t>TCPIP STC 起動時の値</t>
         </is>
       </c>
-      <c r="D16" s="2" t="inlineStr">
+      <c r="E16" s="2" t="inlineStr">
         <is>
           <t>整数</t>
         </is>
       </c>
-      <c r="E16" s="2" t="inlineStr">
+      <c r="F16" s="2" t="inlineStr">
         <is>
           <t>TCPIP STC 再起動 or VARY TCPIP,,OBEYFILE</t>
         </is>
       </c>
-      <c r="F16" s="2" t="inlineStr">
+      <c r="G16" s="2" t="inlineStr">
         <is>
           <t>TCP/IP</t>
         </is>
       </c>
-      <c r="G16" s="2" t="inlineStr">
+      <c r="H16" s="2" t="inlineStr">
         <is>
           <t>cfg-tcpip-profile</t>
         </is>
       </c>
-      <c r="H16" s="2" t="inlineStr">
+      <c r="I16" s="2" t="inlineStr">
         <is>
           <t>S_ZOS_CommServer</t>
         </is>
       </c>
-      <c r="I16" s="2" t="inlineStr">
+      <c r="J16" s="2" t="inlineStr">
         <is>
           <t>同時オープン socket 上限。Web/Server 用途では大きくする必要あり。</t>
         </is>
@@ -8713,40 +9466,45 @@
       </c>
       <c r="B17" s="2" t="inlineStr">
         <is>
+          <t>構成定義</t>
+        </is>
+      </c>
+      <c r="C17" s="2" t="inlineStr">
+        <is>
           <t>SETROPTS コマンド</t>
         </is>
       </c>
-      <c r="C17" s="2" t="inlineStr">
+      <c r="D17" s="2" t="inlineStr">
         <is>
           <t>サイトポリシーにより異なる</t>
         </is>
       </c>
-      <c r="D17" s="2" t="inlineStr">
+      <c r="E17" s="2" t="inlineStr">
         <is>
           <t>PASSWORD(...) / GENERIC(...) / CLASSACT(...) / AUDIT(...) 等</t>
         </is>
       </c>
-      <c r="E17" s="2" t="inlineStr">
+      <c r="F17" s="2" t="inlineStr">
         <is>
           <t>即時</t>
         </is>
       </c>
-      <c r="F17" s="2" t="inlineStr">
+      <c r="G17" s="2" t="inlineStr">
         <is>
           <t>RACF</t>
         </is>
       </c>
-      <c r="G17" s="2" t="inlineStr">
+      <c r="H17" s="2" t="inlineStr">
         <is>
           <t>cfg-racf-permit</t>
         </is>
       </c>
-      <c r="H17" s="2" t="inlineStr">
+      <c r="I17" s="2" t="inlineStr">
         <is>
           <t>S_ZOS_RACF</t>
         </is>
       </c>
-      <c r="I17" s="2" t="inlineStr">
+      <c r="J17" s="2" t="inlineStr">
         <is>
           <t>RACF 全体設定変更コマンド。SETR LIST で現状確認。</t>
         </is>
@@ -8760,40 +9518,45 @@
       </c>
       <c r="B18" s="2" t="inlineStr">
         <is>
+          <t>運用ポリシー</t>
+        </is>
+      </c>
+      <c r="C18" s="2" t="inlineStr">
+        <is>
           <t>RACF SETROPTS PASSWORD(INTERVAL(n))</t>
         </is>
       </c>
-      <c r="C18" s="2" t="inlineStr">
+      <c r="D18" s="2" t="inlineStr">
         <is>
           <t>サイトポリシーで設定（典型 30/60/90 日）</t>
         </is>
       </c>
-      <c r="D18" s="2" t="inlineStr">
+      <c r="E18" s="2" t="inlineStr">
         <is>
           <t>1〜254 日 / 0=無期限</t>
         </is>
       </c>
-      <c r="E18" s="2" t="inlineStr">
+      <c r="F18" s="2" t="inlineStr">
         <is>
           <t>即時</t>
         </is>
       </c>
-      <c r="F18" s="2" t="inlineStr">
+      <c r="G18" s="2" t="inlineStr">
         <is>
           <t>RACF, USERID</t>
         </is>
       </c>
-      <c r="G18" s="2" t="inlineStr">
+      <c r="H18" s="2" t="inlineStr">
         <is>
           <t>cfg-racf-permit</t>
         </is>
       </c>
-      <c r="H18" s="2" t="inlineStr">
+      <c r="I18" s="2" t="inlineStr">
         <is>
           <t>S_ZOS_RACF</t>
         </is>
       </c>
-      <c r="I18" s="2" t="inlineStr">
+      <c r="J18" s="2" t="inlineStr">
         <is>
           <t>ユーザパスワード有効期限。組織のセキュリティポリシーに従い設定。</t>
         </is>
@@ -8807,36 +9570,41 @@
       </c>
       <c r="B19" s="2" t="inlineStr">
         <is>
+          <t>ランタイム</t>
+        </is>
+      </c>
+      <c r="C19" s="2" t="inlineStr">
+        <is>
           <t>CEEPRMxx</t>
         </is>
       </c>
-      <c r="C19" s="2" t="inlineStr">
+      <c r="D19" s="2" t="inlineStr">
         <is>
           <t>サイトにより異なる</t>
         </is>
       </c>
-      <c r="D19" s="2" t="inlineStr">
+      <c r="E19" s="2" t="inlineStr">
         <is>
           <t>Language Environment runtime options</t>
         </is>
       </c>
-      <c r="E19" s="2" t="inlineStr">
+      <c r="F19" s="2" t="inlineStr">
         <is>
           <t>次回 IPL or SET CEE=xx</t>
         </is>
       </c>
-      <c r="F19" s="2" t="inlineStr">
+      <c r="G19" s="2" t="inlineStr">
         <is>
           <t>Language Environment</t>
         </is>
       </c>
-      <c r="G19" s="2" t="inlineStr"/>
-      <c r="H19" s="2" t="inlineStr">
+      <c r="H19" s="2" t="inlineStr"/>
+      <c r="I19" s="2" t="inlineStr">
         <is>
           <t>S_ZOS_LE</t>
         </is>
       </c>
-      <c r="I19" s="2" t="inlineStr">
+      <c r="J19" s="2" t="inlineStr">
         <is>
           <t>LE runtime options（HEAP, STACK, ABTERMENC 等）。COBOL/PL/I/C プログラム実行環境。</t>
         </is>
@@ -8850,40 +9618,45 @@
       </c>
       <c r="B20" s="2" t="inlineStr">
         <is>
+          <t>サイジング</t>
+        </is>
+      </c>
+      <c r="C20" s="2" t="inlineStr">
+        <is>
           <t>IEASYSxx の MAXSPACE</t>
         </is>
       </c>
-      <c r="C20" s="2" t="inlineStr">
+      <c r="D20" s="2" t="inlineStr">
         <is>
           <t>1500M</t>
         </is>
       </c>
-      <c r="D20" s="2" t="inlineStr">
+      <c r="E20" s="2" t="inlineStr">
         <is>
           <t>100M 〜</t>
         </is>
       </c>
-      <c r="E20" s="2" t="inlineStr">
+      <c r="F20" s="2" t="inlineStr">
         <is>
           <t>次回 IPL 時のみ</t>
         </is>
       </c>
-      <c r="F20" s="2" t="inlineStr">
+      <c r="G20" s="2" t="inlineStr">
         <is>
           <t>Auxiliary Storage, PLPA</t>
         </is>
       </c>
-      <c r="G20" s="2" t="inlineStr">
+      <c r="H20" s="2" t="inlineStr">
         <is>
           <t>cfg-parmlib-update</t>
         </is>
       </c>
-      <c r="H20" s="2" t="inlineStr">
+      <c r="I20" s="2" t="inlineStr">
         <is>
           <t>S_ZOS_Init_Tuning</t>
         </is>
       </c>
-      <c r="I20" s="2" t="inlineStr">
+      <c r="J20" s="2" t="inlineStr">
         <is>
           <t>Aux Storage に書き出される SVC dump の最大サイズ。dump 過大化抑止。</t>
         </is>
@@ -8897,40 +9670,45 @@
       </c>
       <c r="B21" s="2" t="inlineStr">
         <is>
+          <t>モード選択</t>
+        </is>
+      </c>
+      <c r="C21" s="2" t="inlineStr">
+        <is>
           <t>IEASYSxx の SCH= オペランド</t>
         </is>
       </c>
-      <c r="C21" s="2" t="inlineStr">
-        <is>
-          <t>00（IEASCH00 を読む）</t>
-        </is>
-      </c>
       <c r="D21" s="2" t="inlineStr">
         <is>
+          <t>00（IEASCH00 メンバを読む。site で複数連結も可）</t>
+        </is>
+      </c>
+      <c r="E21" s="2" t="inlineStr">
+        <is>
           <t>00〜99 の suffix 連結</t>
         </is>
       </c>
-      <c r="E21" s="2" t="inlineStr">
+      <c r="F21" s="2" t="inlineStr">
         <is>
           <t>次回 IPL 時のみ</t>
         </is>
       </c>
-      <c r="F21" s="2" t="inlineStr">
+      <c r="G21" s="2" t="inlineStr">
         <is>
           <t>Subsystem Initialization</t>
         </is>
       </c>
-      <c r="G21" s="2" t="inlineStr">
+      <c r="H21" s="2" t="inlineStr">
         <is>
           <t>cfg-parmlib-update</t>
         </is>
       </c>
-      <c r="H21" s="2" t="inlineStr">
+      <c r="I21" s="2" t="inlineStr">
         <is>
           <t>S_ZOS_Init_Tuning</t>
         </is>
       </c>
-      <c r="I21" s="2" t="inlineStr">
+      <c r="J21" s="2" t="inlineStr">
         <is>
           <t>Schedule（スケジュール）情報。IEASCHxx で program properties 定義。</t>
         </is>

</xml_diff>

<commit_message>
z/OS 3.1 v4: review-fix B+ -> A. P0: 6 virtual-memory headings (SVC/PSA/CSA/ECSA/ESQA/CVT) with independent anchors in 03-glossary; 25 -> 30 use-case count fix in 10-out-of-scope; 3 scenario disclaimers customized (DR/security/PTF) in 11-scenarios. P1: 08/09 matrix tables wrapped in scrollwrap div; CLOCKxx TIMEZONE example E.09 confirmed; image count text normalized to 72. extra.css shared mobile rules with AIX v12.
</commit_message>
<xml_diff>
--- a/docs/products/files/zOS_3.1.xlsx
+++ b/docs/products/files/zOS_3.1.xlsx
@@ -641,7 +641,7 @@
       </c>
       <c r="B11" s="2" t="inlineStr">
         <is>
-          <t>70 件</t>
+          <t>78 件</t>
         </is>
       </c>
       <c r="C11" s="2" t="inlineStr">
@@ -8344,22 +8344,22 @@
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
         <is>
-          <t>Master Catalog (SYS1.NUCLEUS)</t>
+          <t>Master Catalog</t>
         </is>
       </c>
       <c r="B14" s="2" t="inlineStr">
         <is>
-          <t>z/OS 起動時の最初のカタログ。SYS1.* 等のシステムデータセット定義を含む。</t>
+          <t>z/OS 起動時の最初のカタログ。SYS1.* 等のシステムデータセット定義と User Catalog への alias を含む独立 VSAM データセット（命名は通常 SYS1.MASTER.ICFCAT 等）。</t>
         </is>
       </c>
       <c r="C14" s="2" t="inlineStr">
         <is>
-          <t>IDCAMS（DEFINE / DELETE）</t>
+          <t>IDCAMS（DEFINE / DELETE / DEFINE ALIAS）</t>
         </is>
       </c>
       <c r="D14" s="2" t="inlineStr">
         <is>
-          <t>即時</t>
+          <t>即時（カタログ操作）</t>
         </is>
       </c>
       <c r="E14" s="2" t="inlineStr">
@@ -8374,7 +8374,7 @@
       </c>
       <c r="G14" s="2" t="inlineStr">
         <is>
-          <t>Master Catalog 損傷は IPL 失敗の致命傷。alias 経由で User Catalog にチェーン。</t>
+          <t>LOADxx の SYSCAT ステートメントで Master Catalog 名を指定（旧 SYSCATxx メンバ方式は LOADxx に統合済み）。SYS1.NUCLEUS は IPL モジュール格納の PDS であり Master Catalog 自体ではない。Master Catalog 損傷は IPL 失敗の致命傷。</t>
         </is>
       </c>
     </row>
@@ -8534,7 +8534,7 @@
       </c>
       <c r="B19" s="2" t="inlineStr">
         <is>
-          <t>システムクロック・タイムゾーン設定。</t>
+          <t>システムクロック・タイムゾーン設定（TIMEZONE / OPERATOR / ETRMODE 等）。</t>
         </is>
       </c>
       <c r="C19" s="2" t="inlineStr">
@@ -8559,7 +8559,7 @@
       </c>
       <c r="G19" s="2" t="inlineStr">
         <is>
-          <t>TIMEZONE W.09.00.00 等で UTC からの offset 指定（日本は W=west of GMT は誤り、EAST 表記）。</t>
+          <t>TIMEZONE は GMT からの offset を指定。日本（JST = UTC+9）は `TIMEZONE E.09.00.00`（E = East of GMT）。米国東部標準時は `TIMEZONE W.05.00.00`。OPERATOR PROMPT を NO に設定すると IPL 時の日付確認をスキップ。</t>
         </is>
       </c>
     </row>
@@ -9725,7 +9725,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F71"/>
+  <dimension ref="A1:F79"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -11951,6 +11951,254 @@
         </is>
       </c>
       <c r="F71" s="2" t="inlineStr">
+        <is>
+          <t>S_ZOS_MVS_Init</t>
+        </is>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" s="2" t="inlineStr">
+        <is>
+          <t>PSA</t>
+        </is>
+      </c>
+      <c r="B72" s="2" t="inlineStr">
+        <is>
+          <t>仮想記憶</t>
+        </is>
+      </c>
+      <c r="C72" s="2" t="inlineStr">
+        <is>
+          <t>Prefixed Save Area。各 CPU 専用の最下位 8KB 仮想記憶領域（CPU ごとにプレフィックスレジスタで区別）。割込処理用 PSW・レジスタ保管域、CVT へのポインタ等を含む。</t>
+        </is>
+      </c>
+      <c r="D72" s="2" t="inlineStr">
+        <is>
+          <t>CVT, SQA, ASID</t>
+        </is>
+      </c>
+      <c r="E72" s="2" t="inlineStr"/>
+      <c r="F72" s="2" t="inlineStr">
+        <is>
+          <t>S_ZOS_MVS_Init</t>
+        </is>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" s="2" t="inlineStr">
+        <is>
+          <t>CSA</t>
+        </is>
+      </c>
+      <c r="B73" s="2" t="inlineStr">
+        <is>
+          <t>仮想記憶</t>
+        </is>
+      </c>
+      <c r="C73" s="2" t="inlineStr">
+        <is>
+          <t>Common Service Area。全 Address Space で共有される 16MB 境界より下の仮想記憶。サブシステム間共有データに使用。IEASYSxx の CSA= で 1 番目に指定。</t>
+        </is>
+      </c>
+      <c r="D73" s="2" t="inlineStr">
+        <is>
+          <t>ECSA, SQA, IEASYSxx</t>
+        </is>
+      </c>
+      <c r="E73" s="2" t="inlineStr">
+        <is>
+          <t>cfg-parmlib-update</t>
+        </is>
+      </c>
+      <c r="F73" s="2" t="inlineStr">
+        <is>
+          <t>S_ZOS_Init_Tuning</t>
+        </is>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" s="2" t="inlineStr">
+        <is>
+          <t>ECSA</t>
+        </is>
+      </c>
+      <c r="B74" s="2" t="inlineStr">
+        <is>
+          <t>仮想記憶</t>
+        </is>
+      </c>
+      <c r="C74" s="2" t="inlineStr">
+        <is>
+          <t>Extended Common Service Area。16MB 境界より上の CSA。Db2/CICS/MQ 等のサブシステムが多く消費。IEASYSxx の CSA= で 2 番目に指定。</t>
+        </is>
+      </c>
+      <c r="D74" s="2" t="inlineStr">
+        <is>
+          <t>CSA, ESQA, IEASYSxx</t>
+        </is>
+      </c>
+      <c r="E74" s="2" t="inlineStr">
+        <is>
+          <t>cfg-parmlib-update</t>
+        </is>
+      </c>
+      <c r="F74" s="2" t="inlineStr">
+        <is>
+          <t>S_ZOS_Init_Tuning</t>
+        </is>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" s="2" t="inlineStr">
+        <is>
+          <t>SQA</t>
+        </is>
+      </c>
+      <c r="B75" s="2" t="inlineStr">
+        <is>
+          <t>仮想記憶</t>
+        </is>
+      </c>
+      <c r="C75" s="2" t="inlineStr">
+        <is>
+          <t>System Queue Area。z/OS カーネルが使う共有制御ブロック領域（16MB 境界より下）。枯渇すると IPL 失敗・システム停止リスク。IEASYSxx の SQA= で指定。</t>
+        </is>
+      </c>
+      <c r="D75" s="2" t="inlineStr">
+        <is>
+          <t>ESQA, CSA, IEASYSxx</t>
+        </is>
+      </c>
+      <c r="E75" s="2" t="inlineStr">
+        <is>
+          <t>cfg-parmlib-update</t>
+        </is>
+      </c>
+      <c r="F75" s="2" t="inlineStr">
+        <is>
+          <t>S_ZOS_Init_Tuning</t>
+        </is>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" s="2" t="inlineStr">
+        <is>
+          <t>ESQA</t>
+        </is>
+      </c>
+      <c r="B76" s="2" t="inlineStr">
+        <is>
+          <t>仮想記憶</t>
+        </is>
+      </c>
+      <c r="C76" s="2" t="inlineStr">
+        <is>
+          <t>Extended SQA。16MB 境界より上の SQA。Address Space 数増加・Sysplex/Db2 規模拡大とともに増量必要。</t>
+        </is>
+      </c>
+      <c r="D76" s="2" t="inlineStr">
+        <is>
+          <t>SQA, ECSA, IEASYSxx</t>
+        </is>
+      </c>
+      <c r="E76" s="2" t="inlineStr">
+        <is>
+          <t>cfg-parmlib-update</t>
+        </is>
+      </c>
+      <c r="F76" s="2" t="inlineStr">
+        <is>
+          <t>S_ZOS_Init_Tuning</t>
+        </is>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" s="2" t="inlineStr">
+        <is>
+          <t>LPA</t>
+        </is>
+      </c>
+      <c r="B77" s="2" t="inlineStr">
+        <is>
+          <t>仮想記憶</t>
+        </is>
+      </c>
+      <c r="C77" s="2" t="inlineStr">
+        <is>
+          <t>Link Pack Area。z/OS 共通の常駐モジュール領域。PLPA/MLPA/FLPA の 3 種に分類。CLPA で再構築。LPALSTxx でデータセット連結を定義。</t>
+        </is>
+      </c>
+      <c r="D77" s="2" t="inlineStr">
+        <is>
+          <t>CLPA, LPALSTxx</t>
+        </is>
+      </c>
+      <c r="E77" s="2" t="inlineStr">
+        <is>
+          <t>cfg-clpa-ipl</t>
+        </is>
+      </c>
+      <c r="F77" s="2" t="inlineStr">
+        <is>
+          <t>S_ZOS_Init_Tuning</t>
+        </is>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" s="2" t="inlineStr">
+        <is>
+          <t>SVC</t>
+        </is>
+      </c>
+      <c r="B78" s="2" t="inlineStr">
+        <is>
+          <t>仮想記憶</t>
+        </is>
+      </c>
+      <c r="C78" s="2" t="inlineStr">
+        <is>
+          <t>Supervisor Call。問題プログラムから z/OS カーネルサービスを呼び出す機械命令（SVC 番号で識別）。SVC dump, SVC table 等の用語にも登場。SVC dump = SVC 命令で取得するメモリダンプ。</t>
+        </is>
+      </c>
+      <c r="D78" s="2" t="inlineStr">
+        <is>
+          <t>MAXSPACE, SVC dump</t>
+        </is>
+      </c>
+      <c r="E78" s="2" t="inlineStr">
+        <is>
+          <t>inc-svc-dump</t>
+        </is>
+      </c>
+      <c r="F78" s="2" t="inlineStr">
+        <is>
+          <t>S_ZOS_MVS_Diag</t>
+        </is>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" s="2" t="inlineStr">
+        <is>
+          <t>CVT</t>
+        </is>
+      </c>
+      <c r="B79" s="2" t="inlineStr">
+        <is>
+          <t>仮想記憶</t>
+        </is>
+      </c>
+      <c r="C79" s="2" t="inlineStr">
+        <is>
+          <t>Communication Vector Table。z/OS の中核制御ブロック。各種制御ブロック・テーブルへのポインタを集約。PSA 内のオフセットからアクセス可能。</t>
+        </is>
+      </c>
+      <c r="D79" s="2" t="inlineStr">
+        <is>
+          <t>PSA, JESCT, SSCVT</t>
+        </is>
+      </c>
+      <c r="E79" s="2" t="inlineStr"/>
+      <c r="F79" s="2" t="inlineStr">
         <is>
           <t>S_ZOS_MVS_Init</t>
         </is>

</xml_diff>